<commit_message>
Changed the lesson tree file
</commit_message>
<xml_diff>
--- a/data/describe/LessonTree.xlsx
+++ b/data/describe/LessonTree.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Dropbox\OPP_teaching_agent\data\describe\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Dropbox\OOP_new\data\describe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F376BD2-386F-4E3E-835A-3C4FA9250E6A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E23B262A-B38A-4282-BBC9-1992D02CB26D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{01CF3F39-BDE8-4829-BFEC-CEB8AF08EFB3}"/>
   </bookViews>
@@ -193,7 +193,8 @@
     <t>topic</t>
   </si>
   <si>
-    <t>Tell the user, its okay that they do not know the components of the class and provide a brief explanation to the user on what are the key components of a class as used in Object Oriented Programming.</t>
+    <t>Tell the user, its okay that they do not know the components of the class and provide a brief explanation to the user on what are the key components of a class as used in Object Oriented Programming.
+Provide the user with an example of a class and its componets using the C++ syntax and then provide the user with a partial defination of the class and ask the user to compelete it.</t>
   </si>
 </sst>
 </file>
@@ -640,7 +641,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
update the lessonTree file
</commit_message>
<xml_diff>
--- a/data/describe/LessonTree.xlsx
+++ b/data/describe/LessonTree.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Dropbox\OOP_new\data\describe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E23B262A-B38A-4282-BBC9-1992D02CB26D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D9341D8-AE03-41BF-9AE7-A4F601DCC5AF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{01CF3F39-BDE8-4829-BFEC-CEB8AF08EFB3}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Next</t>
   </si>
@@ -43,9 +43,6 @@
   </si>
   <si>
     <t>Classes are templetes for creating objects</t>
-  </si>
-  <si>
-    <t>Check the user definition of a class and use your knowledge of classes in object oriented programming to see if the user answer is correct. If the user answer is correct, tell the user they are right and ask the user to tell you the components of a class in object oriented programming. If the user answer is not correct, tell the user the correct definition of a class in object oriented and ask the user to give you the components of a class in object oriented programming.</t>
   </si>
   <si>
     <t>A class has an object and methods</t>
@@ -195,6 +192,113 @@
   <si>
     <t>Tell the user, its okay that they do not know the components of the class and provide a brief explanation to the user on what are the key components of a class as used in Object Oriented Programming.
 Provide the user with an example of a class and its componets using the C++ syntax and then provide the user with a partial defination of the class and ask the user to compelete it.</t>
+  </si>
+  <si>
+    <t>I don’t know anthing about classes</t>
+  </si>
+  <si>
+    <t>Tell the user that it is okay they don't know anything about classes. Explain to the user what a class is as used in C++ programming and give the user an example of a class and ask the user for another example of a class.</t>
+  </si>
+  <si>
+    <t>An example of a class can be class person or employee</t>
+  </si>
+  <si>
+    <t>I want to learn about inheritence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tell the user, it is great they want to learn about inheritance. Explain to the user what inheritance is according to your knowledge of object-oriented programming. Then ask the user what they know about inheritance and how it is related to inheritance as used in the real day-to-day? </t>
+  </si>
+  <si>
+    <t>Just as in real life classes can inherit the properties of other existing classes</t>
+  </si>
+  <si>
+    <t>Tell the user they are correct and give the user an example of inheritance in object-oriented programming a per the C++ programming language. Then provide the user with a partial example of inheritance and ask the user to complete the example.</t>
+  </si>
+  <si>
+    <t>Check the users answer and show them how that example can be converted into the C++ code. Ask the user to indetify the components of a class.</t>
+  </si>
+  <si>
+    <t>Check the user definition of a class and use your knowledge of classes in object oriented programming to see if the user answer is correct. If the user answer is correct, tell the user they are right and ask the user to tell you the components of a class in object oriented programming. If the user answer is not correct, tell the user the correct definition of a class in object oriented and ask the user to give you an example of a class in object oriented programming.</t>
+  </si>
+  <si>
+    <t>#include &lt;iostream&gt;
+using namespace std;
+// Base class
+class Animal {
+public:
+    void eat() {
+        cout &lt;&lt; "This animal eats food." &lt;&lt; endl;
+    }
+};
+// Derived class
+class Dog : public Animal {
+public:
+    void bark() {
+        cout &lt;&lt; "The dog barks." &lt;&lt; endl;
+    }
+};
+int main() {
+    Dog myDog;
+    // Call function from base class
+    myDog.eat();
+    // Call function from derived class
+    myDog.bark();
+    return 0;
+}</t>
+  </si>
+  <si>
+    <t>Check the user-provided answer if it is correct according to the C++ sytax, congratulate the user for getting it right, then give the user a problem to solve based on the concept,
+If the user's answer is not correct, point to the user, where the problem is and ask the user to try again.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to learn about encasupulation </t>
+  </si>
+  <si>
+    <t>Explain to the user about encapsulation and give an example of encapsulation, then provide the user with an example of encapsulation using the C++ programming language. Then provide the user with a partially solved example and ask the user to complete it.</t>
+  </si>
+  <si>
+    <t>#include &lt;iostream&gt;
+using namespace std;
+class BankAccount {
+private:
+    // Data members are kept private
+    double balance;
+public:
+    // Constructor
+    BankAccount(double initialBalance) {
+        if (initialBalance &gt;= 0)
+            balance = initialBalance;
+        else
+            balance = 0;
+    }
+    // Public method to deposit money
+    void deposit(double amount) {
+        if (amount &gt; 0)
+            balance += amount;
+    }
+    // Public method to withdraw money
+    void withdraw(double amount) {
+        if (amount &gt; 0 &amp;&amp; amount &lt;= balance)
+            balance -= amount;
+        else
+            cout &lt;&lt; "Insufficient funds or invalid amount!" &lt;&lt; endl;
+    }
+    // Public method to check balance
+    double getBalance() {
+        return balance;
+    }
+};
+int main() {
+    BankAccount account(1000);  // Create an account with initial balance
+    account.deposit(500);       // Deposit money
+    account.withdraw(200);      // Withdraw money
+    // Accessing balance via a public method
+    cout &lt;&lt; "Current balance: Ksh " &lt;&lt; account.getBalance() &lt;&lt; endl;
+    return 0;
+}</t>
+  </si>
+  <si>
+    <t>Check the user answer, if it is correct as per your knowledge on oject orieted programming as used in the C++ programming langauge. If it is correct, congragulate the user and give the user a problem to solve on the same concept to solve. If the user answer is not correct, point to the user where the error is, and ask  the user to try again.</t>
   </si>
 </sst>
 </file>
@@ -549,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{097C52EF-578A-428C-82B7-306A5B38F0B5}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="68.81640625" customWidth="1"/>
@@ -562,16 +666,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" t="s">
         <v>19</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>20</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -598,55 +702,111 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="116" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="203" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="145" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>22</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated the LessonTree file
</commit_message>
<xml_diff>
--- a/data/describe/LessonTree.xlsx
+++ b/data/describe/LessonTree.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Dropbox\OOP_new\data\describe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D9341D8-AE03-41BF-9AE7-A4F601DCC5AF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DC4E2B-BC40-48E8-94A0-8C16DE6CBFC6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{01CF3F39-BDE8-4829-BFEC-CEB8AF08EFB3}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Next</t>
   </si>
@@ -299,6 +299,24 @@
   </si>
   <si>
     <t>Check the user answer, if it is correct as per your knowledge on oject orieted programming as used in the C++ programming langauge. If it is correct, congragulate the user and give the user a problem to solve on the same concept to solve. If the user answer is not correct, point to the user where the error is, and ask  the user to try again.</t>
+  </si>
+  <si>
+    <t>I want to learn about constructors and destructors</t>
+  </si>
+  <si>
+    <t>Tell the user it is great that they want to learn about constructors and destructors. Explain to the user what constructors and destructors are in the context of object-oriented programming. Then give the user an example of using the constructors and destructors in object-oriented programming per the C++ programming language. Then provide the user with an incomplete example on constructors and destructors and ask the user to complete it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to learn about polymorphism </t>
+  </si>
+  <si>
+    <t>Tell the user it is great that they want to learn about polymorphism. Explain to the user what polymorphism is in the context of object-oriented programming. Then give the user an example of using polymorphism in object-oriented programming per the C++ programming language. Then provide the user with an incomplete example on polymorphism and ask the user to complete it.</t>
+  </si>
+  <si>
+    <t>I want to learn about access specifiers</t>
+  </si>
+  <si>
+    <t>Tell the user it is great that they want to learn about access specifiers as used in object-oriented programming. Explain to the user what access specifiers are in the context of object-oriented programming. Then give the user an example of using the access specifiers in object-oriented programming per the C++ programming language. Then provide the user with an incomplete example on access specifiers and ask the user to complete it.</t>
   </si>
 </sst>
 </file>
@@ -653,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{097C52EF-578A-428C-82B7-306A5B38F0B5}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="68.81640625" customWidth="1"/>
@@ -809,6 +827,30 @@
         <v>36</v>
       </c>
     </row>
+    <row r="18" spans="1:2" ht="116" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>